<commit_message>
Refresh in-year data for September 2026
</commit_message>
<xml_diff>
--- a/docs/inyear.xlsx
+++ b/docs/inyear.xlsx
@@ -495,14 +495,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Program year 2026-2027. Dashboard snapshot 12-Sep-2026. Built 2026-09-13 11:22 PDT.</t>
+          <t>Program year 2026-2027. Dashboard snapshot 19-Sep-2026. Built 2026-09-20 11:20 PDT.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>290 days remain until 30 June 2027, when these scores become final.</t>
+          <t>283 days remain until 30 June 2027, when these scores become final.</t>
         </is>
       </c>
     </row>
@@ -574,21 +574,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Officer list on time - closes 2026-12-31 (109 days) - 17 clubs short</t>
+          <t xml:space="preserve">   Officer list on time - closes 2026-12-31 (102 days) - 17 clubs short</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Officers trained Nov-Feb - closes 2027-02-28 (168 days) - window opens 2026-11-01</t>
+          <t xml:space="preserve">   Officers trained Nov-Feb - closes 2027-02-28 (161 days) - window opens 2026-11-01</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Renewal dues on time - closes 2027-03-31 (199 days) - 89 clubs short</t>
+          <t xml:space="preserve">   Renewal dues on time - closes 2027-03-31 (192 days) - 80 clubs short</t>
         </is>
       </c>
     </row>
@@ -883,9 +883,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O2" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P2" s="9" t="n">
@@ -1400,9 +1400,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O7" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P7" s="9" t="n">
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>10</v>
@@ -1641,8 +1641,8 @@
       <c r="Y9" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Z9" s="9" t="n">
-        <v>0</v>
+      <c r="Z9" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="AA9" s="10" t="n">
         <v>1</v>
@@ -1676,7 +1676,7 @@
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>10</v>
@@ -1728,8 +1728,8 @@
       <c r="S10" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="T10" s="9" t="n">
-        <v>0</v>
+      <c r="T10" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="U10" s="9" t="n">
         <v>0</v>
@@ -1845,8 +1845,8 @@
       <c r="W11" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X11" s="9" t="n">
-        <v>3</v>
+      <c r="X11" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y11" s="9" t="n">
         <v>0</v>
@@ -1882,7 +1882,7 @@
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" s="6" t="n">
         <v>10</v>
@@ -1934,8 +1934,8 @@
       <c r="S12" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="T12" s="9" t="n">
-        <v>0</v>
+      <c r="T12" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="U12" s="9" t="n">
         <v>0</v>
@@ -2434,9 +2434,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O17" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P17" s="9" t="n">
@@ -2640,9 +2640,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O19" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P19" s="9" t="n">
@@ -3368,7 +3368,7 @@
         <v>2</v>
       </c>
       <c r="Q26" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R26" s="9" t="n">
         <v>0</v>
@@ -3389,7 +3389,7 @@
         <v>0</v>
       </c>
       <c r="X26" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y26" s="9" t="n">
         <v>0</v>
@@ -3750,13 +3750,13 @@
         </is>
       </c>
       <c r="I30" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J30" s="4" t="n">
         <v>23</v>
       </c>
       <c r="K30" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
@@ -3795,7 +3795,7 @@
         <v>0</v>
       </c>
       <c r="V30" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W30" s="9" t="n">
         <v>0</v>
@@ -3841,7 +3841,7 @@
         </is>
       </c>
       <c r="E31" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F31" s="6" t="n">
         <v>10</v>
@@ -3911,8 +3911,8 @@
       <c r="Y31" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Z31" s="9" t="n">
-        <v>0</v>
+      <c r="Z31" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="AA31" s="10" t="n">
         <v>1</v>
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="I35" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J35" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K35" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L35" s="7" t="inlineStr">
         <is>
@@ -4312,7 +4312,7 @@
         <v>0</v>
       </c>
       <c r="V35" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W35" s="9" t="n">
         <v>0</v>
@@ -4595,9 +4595,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O38" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P38" s="9" t="n">
@@ -4968,7 +4968,7 @@
         </is>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F42" s="6" t="n">
         <v>10</v>
@@ -5033,13 +5033,13 @@
         <v>0</v>
       </c>
       <c r="X42" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y42" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Z42" s="9" t="n">
-        <v>0</v>
+      <c r="Z42" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="AA42" s="10" t="n">
         <v>1</v>
@@ -5104,9 +5104,9 @@
           <t>Officer list on time</t>
         </is>
       </c>
-      <c r="O43" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P43" s="9" t="n">
@@ -5619,7 +5619,7 @@
         </is>
       </c>
       <c r="P48" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q48" s="9" t="n">
         <v>1</v>
@@ -5683,7 +5683,7 @@
         </is>
       </c>
       <c r="E49" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F49" s="6" t="n">
         <v>10</v>
@@ -5753,8 +5753,8 @@
       <c r="Y49" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Z49" s="9" t="n">
-        <v>0</v>
+      <c r="Z49" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="AA49" s="10" t="n">
         <v>1</v>
@@ -5924,9 +5924,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O51" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O51" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P51" s="9" t="n">
@@ -6134,16 +6134,16 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O53" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O53" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P53" s="9" t="n">
         <v>1</v>
       </c>
       <c r="Q53" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R53" s="9" t="n">
         <v>0</v>
@@ -7119,7 +7119,7 @@
         </is>
       </c>
       <c r="E63" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F63" s="6" t="n">
         <v>10</v>
@@ -7133,13 +7133,13 @@
         </is>
       </c>
       <c r="I63" s="4" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J63" s="4" t="n">
         <v>52</v>
       </c>
       <c r="K63" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L63" s="4" t="inlineStr">
         <is>
@@ -7177,8 +7177,8 @@
       <c r="U63" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="V63" s="9" t="n">
-        <v>2</v>
+      <c r="V63" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="W63" s="9" t="n">
         <v>0</v>
@@ -7675,9 +7675,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O68" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O68" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P68" s="9" t="n">
@@ -7741,7 +7741,7 @@
         </is>
       </c>
       <c r="E69" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F69" s="6" t="n">
         <v>10</v>
@@ -7811,8 +7811,8 @@
       <c r="Y69" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Z69" s="9" t="n">
-        <v>0</v>
+      <c r="Z69" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="AA69" s="10" t="n">
         <v>1</v>
@@ -8091,9 +8091,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O72" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O72" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P72" s="9" t="n">
@@ -8190,9 +8190,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O73" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O73" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P73" s="9" t="n">
@@ -8563,7 +8563,7 @@
         </is>
       </c>
       <c r="E77" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F77" s="6" t="n">
         <v>10</v>
@@ -8615,8 +8615,8 @@
       <c r="S77" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="T77" s="9" t="n">
-        <v>0</v>
+      <c r="T77" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="U77" s="9" t="n">
         <v>0</v>
@@ -8628,7 +8628,7 @@
         <v>0</v>
       </c>
       <c r="X77" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y77" s="9" t="n">
         <v>0</v>
@@ -9107,9 +9107,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O82" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O82" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P82" s="9" t="n">
@@ -9418,9 +9418,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O85" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O85" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P85" s="9" t="n">
@@ -9523,9 +9523,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O86" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O86" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P86" s="9" t="n">
@@ -9589,7 +9589,7 @@
         </is>
       </c>
       <c r="E87" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F87" s="6" t="n">
         <v>10</v>
@@ -9659,8 +9659,8 @@
       <c r="Y87" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Z87" s="9" t="n">
-        <v>0</v>
+      <c r="Z87" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="AA87" s="10" t="n">
         <v>1</v>
@@ -9931,9 +9931,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O90" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O90" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P90" s="9" t="n">
@@ -10098,7 +10098,7 @@
         </is>
       </c>
       <c r="E92" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F92" s="6" t="n">
         <v>10</v>
@@ -10133,9 +10133,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O92" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O92" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P92" s="9" t="n">
@@ -10150,11 +10150,11 @@
       <c r="S92" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="T92" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="U92" s="9" t="n">
-        <v>0</v>
+      <c r="T92" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="U92" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="V92" s="9" t="n">
         <v>2</v>
@@ -10203,7 +10203,7 @@
         </is>
       </c>
       <c r="E93" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F93" s="6" t="n">
         <v>10</v>
@@ -10252,8 +10252,8 @@
       <c r="R93" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="S93" s="9" t="n">
-        <v>1</v>
+      <c r="S93" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="T93" s="10" t="n">
         <v>1</v>
@@ -10858,7 +10858,7 @@
         </is>
       </c>
       <c r="P99" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q99" s="9" t="n">
         <v>0</v>
@@ -11068,7 +11068,7 @@
         </is>
       </c>
       <c r="P101" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q101" s="9" t="n">
         <v>1</v>
@@ -11233,7 +11233,7 @@
         </is>
       </c>
       <c r="E103" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F103" s="6" t="n">
         <v>10</v>
@@ -11273,8 +11273,8 @@
           <t>submitted</t>
         </is>
       </c>
-      <c r="P103" s="9" t="n">
-        <v>2</v>
+      <c r="P103" s="10" t="n">
+        <v>5</v>
       </c>
       <c r="Q103" s="9" t="n">
         <v>1</v>
@@ -11443,7 +11443,7 @@
         </is>
       </c>
       <c r="E105" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F105" s="6" t="n">
         <v>10</v>
@@ -11478,16 +11478,16 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O105" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O105" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P105" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Q105" s="9" t="n">
-        <v>0</v>
+      <c r="Q105" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="R105" s="9" t="n">
         <v>0</v>
@@ -11680,9 +11680,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O107" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O107" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P107" s="9" t="n">
@@ -11746,7 +11746,7 @@
         </is>
       </c>
       <c r="E108" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F108" s="6" t="n">
         <v>10</v>
@@ -11781,9 +11781,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O108" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O108" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P108" s="9" t="n">
@@ -11795,8 +11795,8 @@
       <c r="R108" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="S108" s="9" t="n">
-        <v>1</v>
+      <c r="S108" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="T108" s="10" t="n">
         <v>1</v>
@@ -11886,9 +11886,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O109" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O109" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P109" s="9" t="n">
@@ -11991,9 +11991,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O110" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O110" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P110" s="9" t="n">
@@ -12071,13 +12071,13 @@
         </is>
       </c>
       <c r="I111" s="4" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="J111" s="4" t="n">
         <v>25</v>
       </c>
       <c r="K111" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L111" s="4" t="inlineStr">
         <is>
@@ -12119,7 +12119,7 @@
         <v>4</v>
       </c>
       <c r="W111" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X111" s="10" t="n">
         <v>7</v>
@@ -12197,9 +12197,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O112" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O112" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P112" s="9" t="n">
@@ -12574,7 +12574,7 @@
         </is>
       </c>
       <c r="E116" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F116" s="6" t="n">
         <v>10</v>
@@ -12609,9 +12609,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O116" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O116" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P116" s="9" t="n">
@@ -12644,8 +12644,8 @@
       <c r="Y116" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Z116" s="9" t="n">
-        <v>0</v>
+      <c r="Z116" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="AA116" s="10" t="n">
         <v>1</v>
@@ -12916,9 +12916,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O119" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O119" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P119" s="9" t="n">
@@ -13423,9 +13423,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O124" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O124" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P124" s="9" t="n">
@@ -13489,7 +13489,7 @@
         </is>
       </c>
       <c r="E125" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F125" s="6" t="n">
         <v>10</v>
@@ -13533,7 +13533,7 @@
         <v>0</v>
       </c>
       <c r="Q125" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R125" s="9" t="n">
         <v>0</v>
@@ -13541,8 +13541,8 @@
       <c r="S125" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="T125" s="9" t="n">
-        <v>0</v>
+      <c r="T125" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="U125" s="9" t="n">
         <v>0</v>
@@ -13911,13 +13911,13 @@
         </is>
       </c>
       <c r="I129" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J129" s="4" t="n">
         <v>6</v>
       </c>
       <c r="K129" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L129" s="7" t="inlineStr">
         <is>
@@ -13956,7 +13956,7 @@
         <v>0</v>
       </c>
       <c r="V129" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W129" s="9" t="n">
         <v>0</v>
@@ -13998,7 +13998,7 @@
         </is>
       </c>
       <c r="E130" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F130" s="6" t="n">
         <v>10</v>
@@ -14048,13 +14048,13 @@
         <v>0</v>
       </c>
       <c r="S130" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T130" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="U130" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="T130" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="U130" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="V130" s="10" t="n">
         <v>4</v>
@@ -14245,7 +14245,7 @@
         </is>
       </c>
       <c r="P132" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q132" s="9" t="n">
         <v>0</v>
@@ -14410,7 +14410,7 @@
         </is>
       </c>
       <c r="E134" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F134" s="6" t="n">
         <v>10</v>
@@ -14445,9 +14445,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O134" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O134" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P134" s="9" t="n">
@@ -14460,10 +14460,10 @@
         <v>0</v>
       </c>
       <c r="S134" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T134" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="T134" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="U134" s="9" t="n">
         <v>0</v>
@@ -14475,7 +14475,7 @@
         <v>0</v>
       </c>
       <c r="X134" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y134" s="9" t="n">
         <v>0</v>
@@ -14515,7 +14515,7 @@
         </is>
       </c>
       <c r="E135" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F135" s="6" t="n">
         <v>10</v>
@@ -14550,9 +14550,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O135" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O135" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P135" s="9" t="n">
@@ -14585,8 +14585,8 @@
       <c r="Y135" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Z135" s="9" t="n">
-        <v>0</v>
+      <c r="Z135" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="AA135" s="10" t="n">
         <v>1</v>
@@ -14861,9 +14861,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O138" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O138" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P138" s="9" t="n">
@@ -15174,7 +15174,7 @@
         </is>
       </c>
       <c r="P141" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q141" s="9" t="n">
         <v>0</v>
@@ -15610,7 +15610,7 @@
         <v>0</v>
       </c>
       <c r="X145" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y145" s="9" t="n">
         <v>0</v>
@@ -15715,7 +15715,7 @@
         <v>0</v>
       </c>
       <c r="X146" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y146" s="9" t="n">
         <v>0</v>
@@ -15895,9 +15895,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O148" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O148" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P148" s="9" t="n">
@@ -16215,7 +16215,7 @@
         <v>0</v>
       </c>
       <c r="Q151" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R151" s="9" t="n">
         <v>0</v>
@@ -16418,7 +16418,7 @@
         </is>
       </c>
       <c r="P153" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q153" s="9" t="n">
         <v>1</v>
@@ -17047,7 +17047,7 @@
         <v>1</v>
       </c>
       <c r="Q159" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R159" s="9" t="n">
         <v>0</v>
@@ -17559,9 +17559,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O164" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O164" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P164" s="9" t="n">
@@ -17993,7 +17993,7 @@
         <v>0</v>
       </c>
       <c r="X168" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Y168" s="9" t="n">
         <v>0</v>
@@ -18202,8 +18202,8 @@
       <c r="W170" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="X170" s="9" t="n">
-        <v>3</v>
+      <c r="X170" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Y170" s="9" t="n">
         <v>0</v>
@@ -18390,7 +18390,7 @@
         <v>0</v>
       </c>
       <c r="S172" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T172" s="10" t="n">
         <v>1</v>
@@ -18476,9 +18476,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O173" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O173" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P173" s="9" t="n">
@@ -18684,7 +18684,7 @@
         </is>
       </c>
       <c r="P175" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q175" s="9" t="n">
         <v>0</v>
@@ -18853,7 +18853,7 @@
         </is>
       </c>
       <c r="E177" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F177" s="6" t="n">
         <v>10</v>
@@ -18867,13 +18867,13 @@
         </is>
       </c>
       <c r="I177" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J177" s="4" t="n">
         <v>6</v>
       </c>
       <c r="K177" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L177" s="7" t="inlineStr">
         <is>
@@ -18912,7 +18912,7 @@
         <v>0</v>
       </c>
       <c r="V177" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W177" s="9" t="n">
         <v>0</v>
@@ -18923,8 +18923,8 @@
       <c r="Y177" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Z177" s="9" t="n">
-        <v>0</v>
+      <c r="Z177" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="AA177" s="10" t="n">
         <v>1</v>
@@ -19073,13 +19073,13 @@
         </is>
       </c>
       <c r="I179" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J179" s="4" t="n">
         <v>21</v>
       </c>
       <c r="K179" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L179" s="4" t="inlineStr">
         <is>
@@ -19118,7 +19118,7 @@
         <v>1</v>
       </c>
       <c r="V179" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W179" s="9" t="n">
         <v>0</v>
@@ -19304,9 +19304,9 @@
           <t>Officers trained Nov-Feb</t>
         </is>
       </c>
-      <c r="O181" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O181" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P181" s="9" t="n">
@@ -19409,9 +19409,9 @@
           <t>Officer list on time</t>
         </is>
       </c>
-      <c r="O182" s="7" t="inlineStr">
-        <is>
-          <t>not yet</t>
+      <c r="O182" s="4" t="inlineStr">
+        <is>
+          <t>submitted</t>
         </is>
       </c>
       <c r="P182" s="9" t="n">
@@ -19778,7 +19778,7 @@
         <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -19811,7 +19811,7 @@
         <v>5</v>
       </c>
       <c r="D4" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
@@ -19943,7 +19943,7 @@
         <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -20042,7 +20042,7 @@
         <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -20075,7 +20075,7 @@
         <v>4</v>
       </c>
       <c r="D12" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
@@ -20174,7 +20174,7 @@
         <v>5</v>
       </c>
       <c r="D15" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -20207,7 +20207,7 @@
         <v>5</v>
       </c>
       <c r="D16" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -20273,7 +20273,7 @@
         <v>7</v>
       </c>
       <c r="D18" t="n">
-        <v>0.29</v>
+        <v>0.43</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -20339,7 +20339,7 @@
         <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -20372,7 +20372,7 @@
         <v>5</v>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -20438,7 +20438,7 @@
         <v>6</v>
       </c>
       <c r="D23" t="n">
-        <v>1.17</v>
+        <v>1.5</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -20471,7 +20471,7 @@
         <v>7</v>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>1.14</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -20504,7 +20504,7 @@
         <v>4</v>
       </c>
       <c r="D25" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -20570,7 +20570,7 @@
         <v>5</v>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -20603,13 +20603,13 @@
         <v>5</v>
       </c>
       <c r="D28" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -20636,7 +20636,7 @@
         <v>5</v>
       </c>
       <c r="D29" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
@@ -20933,7 +20933,7 @@
         <v>5</v>
       </c>
       <c r="D38" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Refresh in-year data for October 2026
</commit_message>
<xml_diff>
--- a/docs/inyear.xlsx
+++ b/docs/inyear.xlsx
@@ -495,14 +495,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Program year 2026-2027. Dashboard snapshot 3-Oct-2026. Built 2026-10-04 11:51 PDT.</t>
+          <t>Program year 2026-2027. Dashboard snapshot 10-Oct-2026. Built 2026-10-11 12:46 PDT.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>269 days remain until 30 June 2027, when these scores become final.</t>
+          <t>262 days remain until 30 June 2027, when these scores become final.</t>
         </is>
       </c>
     </row>
@@ -574,21 +574,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Officer list on time - closes 2026-12-31 (88 days) - 17 clubs short</t>
+          <t xml:space="preserve">   Officer list on time - closes 2026-12-31 (81 days) - 17 clubs short</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Officers trained Nov-Feb - closes 2027-02-28 (147 days) - window opens 2026-11-01</t>
+          <t xml:space="preserve">   Officers trained Nov-Feb - closes 2027-02-28 (140 days) - window opens 2026-11-01</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Renewal dues on time - closes 2027-03-31 (178 days) - 38 clubs short</t>
+          <t xml:space="preserve">   Renewal dues on time - closes 2027-03-31 (171 days) - 37 clubs short</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="J2" s="4" t="n">
         <v>13</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>1</v>
+        <v>-5</v>
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
@@ -963,17 +963,17 @@
         </is>
       </c>
       <c r="I3" s="4" t="n">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="J3" s="4" t="n">
         <v>30</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-13</v>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M3" s="8" t="n">
@@ -1169,13 +1169,13 @@
         </is>
       </c>
       <c r="I5" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="J5" s="4" t="n">
         <v>25</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
@@ -1274,13 +1274,13 @@
         </is>
       </c>
       <c r="I6" s="4" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>10</v>
@@ -1379,17 +1379,17 @@
         </is>
       </c>
       <c r="I7" s="4" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="J7" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-4</v>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M7" s="8" t="n">
@@ -1415,13 +1415,13 @@
         <v>0</v>
       </c>
       <c r="S7" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="U7" s="9" t="n">
-        <v>0</v>
+      <c r="U7" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="V7" s="9" t="n">
         <v>2</v>
@@ -1484,13 +1484,13 @@
         </is>
       </c>
       <c r="I8" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>10</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
@@ -1585,17 +1585,17 @@
         </is>
       </c>
       <c r="I9" s="4" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="J9" s="4" t="n">
         <v>25</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-8</v>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M9" s="8" t="n">
@@ -1633,7 +1633,7 @@
         <v>4</v>
       </c>
       <c r="W9" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X9" s="10" t="n">
         <v>5</v>
@@ -1690,17 +1690,17 @@
         </is>
       </c>
       <c r="I10" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>18</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>1</v>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M10" s="8" t="n">
@@ -1795,13 +1795,13 @@
         </is>
       </c>
       <c r="I11" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J11" s="4" t="n">
         <v>8</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
@@ -1840,7 +1840,7 @@
         <v>0</v>
       </c>
       <c r="V11" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W11" s="9" t="n">
         <v>0</v>
@@ -1896,17 +1896,17 @@
         </is>
       </c>
       <c r="I12" s="4" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>21</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-9</v>
+      </c>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M12" s="8" t="n">
@@ -2001,13 +2001,13 @@
         </is>
       </c>
       <c r="I13" s="4" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="J13" s="4" t="n">
         <v>14</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
@@ -2046,7 +2046,7 @@
         <v>0</v>
       </c>
       <c r="V13" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W13" s="9" t="n">
         <v>0</v>
@@ -2102,13 +2102,13 @@
         </is>
       </c>
       <c r="I14" s="4" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>15</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="L14" s="7" t="inlineStr">
         <is>
@@ -2138,7 +2138,7 @@
         <v>0</v>
       </c>
       <c r="S14" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T14" s="10" t="n">
         <v>1</v>
@@ -2308,13 +2308,13 @@
         </is>
       </c>
       <c r="I16" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J16" s="4" t="n">
         <v>14</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
@@ -2353,7 +2353,7 @@
         <v>0</v>
       </c>
       <c r="V16" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W16" s="9" t="n">
         <v>0</v>
@@ -2413,13 +2413,13 @@
         </is>
       </c>
       <c r="I17" s="4" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="J17" s="4" t="n">
         <v>33</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>2</v>
+        <v>-5</v>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
@@ -2455,10 +2455,10 @@
         <v>1</v>
       </c>
       <c r="U17" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V17" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W17" s="9" t="n">
         <v>0</v>
@@ -2518,13 +2518,13 @@
         </is>
       </c>
       <c r="I18" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="L18" s="7" t="inlineStr">
         <is>
@@ -2619,13 +2619,13 @@
         </is>
       </c>
       <c r="I19" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J19" s="4" t="n">
         <v>9</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="L19" s="7" t="inlineStr">
         <is>
@@ -2720,17 +2720,17 @@
         </is>
       </c>
       <c r="I20" s="4" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>25</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-10</v>
+      </c>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M20" s="8" t="n">
@@ -2750,7 +2750,7 @@
         <v>1</v>
       </c>
       <c r="Q20" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R20" s="9" t="n">
         <v>0</v>
@@ -2825,13 +2825,13 @@
         </is>
       </c>
       <c r="I21" s="4" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="J21" s="4" t="n">
         <v>17</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>1</v>
+        <v>-7</v>
       </c>
       <c r="L21" s="7" t="inlineStr">
         <is>
@@ -2870,7 +2870,7 @@
         <v>0</v>
       </c>
       <c r="V21" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W21" s="9" t="n">
         <v>0</v>
@@ -3132,17 +3132,17 @@
         </is>
       </c>
       <c r="I24" s="4" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="J24" s="4" t="n">
         <v>21</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-10</v>
+      </c>
+      <c r="L24" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M24" s="8" t="n">
@@ -3338,13 +3338,13 @@
         </is>
       </c>
       <c r="I26" s="4" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="J26" s="4" t="n">
         <v>18</v>
       </c>
       <c r="K26" s="4" t="n">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="L26" s="7" t="inlineStr">
         <is>
@@ -3443,13 +3443,13 @@
         </is>
       </c>
       <c r="I27" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J27" s="4" t="n">
         <v>8</v>
       </c>
       <c r="K27" s="4" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="L27" s="7" t="inlineStr">
         <is>
@@ -3544,13 +3544,13 @@
         </is>
       </c>
       <c r="I28" s="4" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J28" s="4" t="n">
         <v>13</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="L28" s="7" t="inlineStr">
         <is>
@@ -3645,17 +3645,17 @@
         </is>
       </c>
       <c r="I29" s="4" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="J29" s="4" t="n">
         <v>27</v>
       </c>
       <c r="K29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-10</v>
+      </c>
+      <c r="L29" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M29" s="8" t="n">
@@ -3690,7 +3690,7 @@
         <v>0</v>
       </c>
       <c r="V29" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W29" s="9" t="n">
         <v>0</v>
@@ -3750,17 +3750,17 @@
         </is>
       </c>
       <c r="I30" s="4" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="J30" s="4" t="n">
         <v>23</v>
       </c>
       <c r="K30" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L30" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-8</v>
+      </c>
+      <c r="L30" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M30" s="8" t="n">
@@ -3855,13 +3855,13 @@
         </is>
       </c>
       <c r="I31" s="4" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="J31" s="4" t="n">
         <v>14</v>
       </c>
       <c r="K31" s="4" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="L31" s="7" t="inlineStr">
         <is>
@@ -3960,13 +3960,13 @@
         </is>
       </c>
       <c r="I32" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J32" s="4" t="n">
         <v>8</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="L32" s="7" t="inlineStr">
         <is>
@@ -4061,17 +4061,17 @@
         </is>
       </c>
       <c r="I33" s="4" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="J33" s="4" t="n">
         <v>28</v>
       </c>
       <c r="K33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L33" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-12</v>
+      </c>
+      <c r="L33" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M33" s="8" t="n">
@@ -4166,13 +4166,13 @@
         </is>
       </c>
       <c r="I34" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="J34" s="4" t="n">
         <v>14</v>
       </c>
       <c r="K34" s="4" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="L34" s="7" t="inlineStr">
         <is>
@@ -4211,7 +4211,7 @@
         <v>0</v>
       </c>
       <c r="V34" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W34" s="9" t="n">
         <v>0</v>
@@ -4267,13 +4267,13 @@
         </is>
       </c>
       <c r="I35" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J35" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K35" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L35" s="7" t="inlineStr">
         <is>
@@ -4312,7 +4312,7 @@
         <v>0</v>
       </c>
       <c r="V35" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W35" s="9" t="n">
         <v>0</v>
@@ -4368,13 +4368,13 @@
         </is>
       </c>
       <c r="I36" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="J36" s="4" t="n">
         <v>14</v>
       </c>
       <c r="K36" s="4" t="n">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="L36" s="7" t="inlineStr">
         <is>
@@ -4413,7 +4413,7 @@
         <v>0</v>
       </c>
       <c r="V36" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W36" s="9" t="n">
         <v>0</v>
@@ -4574,17 +4574,17 @@
         </is>
       </c>
       <c r="I38" s="4" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="J38" s="4" t="n">
         <v>25</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L38" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-8</v>
+      </c>
+      <c r="L38" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M38" s="8" t="n">
@@ -4679,13 +4679,13 @@
         </is>
       </c>
       <c r="I39" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J39" s="4" t="n">
         <v>13</v>
       </c>
       <c r="K39" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L39" s="7" t="inlineStr">
         <is>
@@ -4780,13 +4780,13 @@
         </is>
       </c>
       <c r="I40" s="4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J40" s="4" t="n">
         <v>8</v>
       </c>
       <c r="K40" s="4" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="L40" s="7" t="inlineStr">
         <is>
@@ -4881,17 +4881,17 @@
         </is>
       </c>
       <c r="I41" s="4" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="J41" s="4" t="n">
         <v>21</v>
       </c>
       <c r="K41" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="L41" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-6</v>
+      </c>
+      <c r="L41" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M41" s="8" t="n">
@@ -4982,13 +4982,13 @@
         </is>
       </c>
       <c r="I42" s="4" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J42" s="4" t="n">
         <v>15</v>
       </c>
       <c r="K42" s="4" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="L42" s="7" t="inlineStr">
         <is>
@@ -5009,7 +5009,7 @@
         </is>
       </c>
       <c r="P42" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q42" s="9" t="n">
         <v>1</v>
@@ -5018,7 +5018,7 @@
         <v>0</v>
       </c>
       <c r="S42" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T42" s="9" t="n">
         <v>0</v>
@@ -5083,13 +5083,13 @@
         </is>
       </c>
       <c r="I43" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J43" s="4" t="n">
         <v>10</v>
       </c>
       <c r="K43" s="4" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="L43" s="7" t="inlineStr">
         <is>
@@ -5128,7 +5128,7 @@
         <v>0</v>
       </c>
       <c r="V43" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W43" s="9" t="n">
         <v>0</v>
@@ -5184,13 +5184,13 @@
         </is>
       </c>
       <c r="I44" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="J44" s="4" t="n">
         <v>15</v>
       </c>
       <c r="K44" s="4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="L44" s="7" t="inlineStr">
         <is>
@@ -5271,7 +5271,7 @@
         </is>
       </c>
       <c r="E45" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F45" s="6" t="n">
         <v>10</v>
@@ -5285,13 +5285,13 @@
         </is>
       </c>
       <c r="I45" s="4" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="J45" s="4" t="n">
         <v>30</v>
       </c>
       <c r="K45" s="4" t="n">
-        <v>1</v>
+        <v>-9</v>
       </c>
       <c r="L45" s="4" t="inlineStr">
         <is>
@@ -5323,14 +5323,14 @@
       <c r="S45" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="T45" s="9" t="n">
-        <v>0</v>
+      <c r="T45" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="U45" s="9" t="n">
         <v>0</v>
       </c>
       <c r="V45" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W45" s="9" t="n">
         <v>0</v>
@@ -5390,17 +5390,17 @@
         </is>
       </c>
       <c r="I46" s="4" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="J46" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K46" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L46" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-6</v>
+      </c>
+      <c r="L46" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M46" s="8" t="n">
@@ -5491,13 +5491,13 @@
         </is>
       </c>
       <c r="I47" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="J47" s="4" t="n">
         <v>14</v>
       </c>
       <c r="K47" s="4" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="L47" s="7" t="inlineStr">
         <is>
@@ -5592,13 +5592,13 @@
         </is>
       </c>
       <c r="I48" s="4" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="J48" s="4" t="n">
         <v>27</v>
       </c>
       <c r="K48" s="4" t="n">
-        <v>0</v>
+        <v>-7</v>
       </c>
       <c r="L48" s="4" t="inlineStr">
         <is>
@@ -5697,13 +5697,13 @@
         </is>
       </c>
       <c r="I49" s="4" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="J49" s="4" t="n">
         <v>15</v>
       </c>
       <c r="K49" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L49" s="7" t="inlineStr">
         <is>
@@ -5798,13 +5798,13 @@
         </is>
       </c>
       <c r="I50" s="4" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="J50" s="4" t="n">
         <v>15</v>
       </c>
       <c r="K50" s="4" t="n">
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="L50" s="7" t="inlineStr">
         <is>
@@ -5903,17 +5903,17 @@
         </is>
       </c>
       <c r="I51" s="4" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="J51" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K51" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L51" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-9</v>
+      </c>
+      <c r="L51" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M51" s="8" t="n">
@@ -6008,13 +6008,13 @@
         </is>
       </c>
       <c r="I52" s="4" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="J52" s="4" t="n">
         <v>12</v>
       </c>
       <c r="K52" s="4" t="n">
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="L52" s="7" t="inlineStr">
         <is>
@@ -6113,17 +6113,17 @@
         </is>
       </c>
       <c r="I53" s="4" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="J53" s="4" t="n">
         <v>21</v>
       </c>
       <c r="K53" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L53" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-9</v>
+      </c>
+      <c r="L53" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M53" s="8" t="n">
@@ -6218,17 +6218,17 @@
         </is>
       </c>
       <c r="I54" s="4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="J54" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K54" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L54" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-5</v>
+      </c>
+      <c r="L54" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M54" s="8" t="n">
@@ -6309,7 +6309,7 @@
         </is>
       </c>
       <c r="E55" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F55" s="6" t="n">
         <v>10</v>
@@ -6323,13 +6323,13 @@
         </is>
       </c>
       <c r="I55" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J55" s="4" t="n">
         <v>8</v>
       </c>
       <c r="K55" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L55" s="7" t="inlineStr">
         <is>
@@ -6367,8 +6367,8 @@
       <c r="U55" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="V55" s="9" t="n">
-        <v>1</v>
+      <c r="V55" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="W55" s="9" t="n">
         <v>0</v>
@@ -6424,13 +6424,13 @@
         </is>
       </c>
       <c r="I56" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="J56" s="4" t="n">
         <v>15</v>
       </c>
       <c r="K56" s="4" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="L56" s="7" t="inlineStr">
         <is>
@@ -6451,7 +6451,7 @@
         </is>
       </c>
       <c r="P56" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q56" s="9" t="n">
         <v>1</v>
@@ -6511,7 +6511,7 @@
         </is>
       </c>
       <c r="E57" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F57" s="6" t="n">
         <v>10</v>
@@ -6525,13 +6525,13 @@
         </is>
       </c>
       <c r="I57" s="4" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="J57" s="4" t="n">
         <v>36</v>
       </c>
       <c r="K57" s="4" t="n">
-        <v>2</v>
+        <v>-8</v>
       </c>
       <c r="L57" s="4" t="inlineStr">
         <is>
@@ -6569,8 +6569,8 @@
       <c r="U57" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="V57" s="9" t="n">
-        <v>2</v>
+      <c r="V57" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="W57" s="9" t="n">
         <v>0</v>
@@ -6630,13 +6630,13 @@
         </is>
       </c>
       <c r="I58" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J58" s="4" t="n">
         <v>12</v>
       </c>
       <c r="K58" s="4" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="L58" s="7" t="inlineStr">
         <is>
@@ -6731,13 +6731,13 @@
         </is>
       </c>
       <c r="I59" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J59" s="4" t="n">
         <v>22</v>
       </c>
       <c r="K59" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L59" s="4" t="inlineStr">
         <is>
@@ -6776,7 +6776,7 @@
         <v>0</v>
       </c>
       <c r="V59" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W59" s="9" t="n">
         <v>0</v>
@@ -6830,13 +6830,13 @@
         </is>
       </c>
       <c r="I60" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J60" s="4" t="n">
         <v>10</v>
       </c>
       <c r="K60" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L60" s="7" t="inlineStr">
         <is>
@@ -6931,13 +6931,13 @@
         </is>
       </c>
       <c r="I61" s="4" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="J61" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K61" s="4" t="n">
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="L61" s="7" t="inlineStr">
         <is>
@@ -7032,13 +7032,13 @@
         </is>
       </c>
       <c r="I62" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J62" s="4" t="n">
         <v>9</v>
       </c>
       <c r="K62" s="4" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="L62" s="7" t="inlineStr">
         <is>
@@ -7133,13 +7133,13 @@
         </is>
       </c>
       <c r="I63" s="4" t="n">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="J63" s="4" t="n">
         <v>52</v>
       </c>
       <c r="K63" s="4" t="n">
-        <v>4</v>
+        <v>-18</v>
       </c>
       <c r="L63" s="4" t="inlineStr">
         <is>
@@ -7181,7 +7181,7 @@
         <v>4</v>
       </c>
       <c r="W63" s="9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X63" s="10" t="n">
         <v>7</v>
@@ -7238,13 +7238,13 @@
         </is>
       </c>
       <c r="I64" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J64" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K64" s="4" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="L64" s="7" t="inlineStr">
         <is>
@@ -7339,13 +7339,13 @@
         </is>
       </c>
       <c r="I65" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J65" s="4" t="n">
         <v>12</v>
       </c>
       <c r="K65" s="4" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="L65" s="7" t="inlineStr">
         <is>
@@ -7444,17 +7444,17 @@
         </is>
       </c>
       <c r="I66" s="4" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="J66" s="4" t="n">
         <v>22</v>
       </c>
       <c r="K66" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L66" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-5</v>
+      </c>
+      <c r="L66" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M66" s="8" t="n">
@@ -7471,7 +7471,7 @@
         </is>
       </c>
       <c r="P66" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q66" s="9" t="n">
         <v>0</v>
@@ -7549,13 +7549,13 @@
         </is>
       </c>
       <c r="I67" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="J67" s="4" t="n">
         <v>14</v>
       </c>
       <c r="K67" s="4" t="n">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="L67" s="7" t="inlineStr">
         <is>
@@ -7585,7 +7585,7 @@
         <v>0</v>
       </c>
       <c r="S67" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T67" s="9" t="n">
         <v>0</v>
@@ -7594,7 +7594,7 @@
         <v>0</v>
       </c>
       <c r="V67" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W67" s="9" t="n">
         <v>0</v>
@@ -7654,13 +7654,13 @@
         </is>
       </c>
       <c r="I68" s="4" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="J68" s="4" t="n">
         <v>16</v>
       </c>
       <c r="K68" s="4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="L68" s="7" t="inlineStr">
         <is>
@@ -7755,13 +7755,13 @@
         </is>
       </c>
       <c r="I69" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J69" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K69" s="4" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="L69" s="7" t="inlineStr">
         <is>
@@ -7860,17 +7860,17 @@
         </is>
       </c>
       <c r="I70" s="4" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="J70" s="4" t="n">
         <v>23</v>
       </c>
       <c r="K70" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L70" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-23</v>
+      </c>
+      <c r="L70" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M70" s="8" t="n">
@@ -7965,13 +7965,13 @@
         </is>
       </c>
       <c r="I71" s="4" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="J71" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K71" s="4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L71" s="4" t="inlineStr">
         <is>
@@ -8155,7 +8155,7 @@
         </is>
       </c>
       <c r="E73" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F73" s="6" t="n">
         <v>10</v>
@@ -8213,11 +8213,11 @@
       <c r="U73" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="V73" s="9" t="n">
-        <v>3</v>
+      <c r="V73" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="W73" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X73" s="10" t="n">
         <v>5</v>
@@ -8270,13 +8270,13 @@
         </is>
       </c>
       <c r="I74" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J74" s="4" t="n">
         <v>9</v>
       </c>
       <c r="K74" s="4" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="L74" s="7" t="inlineStr">
         <is>
@@ -8357,7 +8357,7 @@
         </is>
       </c>
       <c r="E75" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F75" s="6" t="n">
         <v>10</v>
@@ -8371,13 +8371,13 @@
         </is>
       </c>
       <c r="I75" s="4" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="J75" s="4" t="n">
         <v>39</v>
       </c>
       <c r="K75" s="4" t="n">
-        <v>3</v>
+        <v>-17</v>
       </c>
       <c r="L75" s="4" t="inlineStr">
         <is>
@@ -8407,7 +8407,7 @@
         <v>0</v>
       </c>
       <c r="S75" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T75" s="9" t="n">
         <v>0</v>
@@ -8415,11 +8415,11 @@
       <c r="U75" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="V75" s="9" t="n">
-        <v>3</v>
+      <c r="V75" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="W75" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X75" s="10" t="n">
         <v>7</v>
@@ -8476,13 +8476,13 @@
         </is>
       </c>
       <c r="I76" s="4" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="J76" s="4" t="n">
         <v>19</v>
       </c>
       <c r="K76" s="4" t="n">
-        <v>0</v>
+        <v>-11</v>
       </c>
       <c r="L76" s="7" t="inlineStr">
         <is>
@@ -8577,17 +8577,17 @@
         </is>
       </c>
       <c r="I77" s="4" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="J77" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K77" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L77" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-6</v>
+      </c>
+      <c r="L77" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M77" s="8" t="n">
@@ -8783,13 +8783,13 @@
         </is>
       </c>
       <c r="I79" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J79" s="4" t="n">
         <v>12</v>
       </c>
       <c r="K79" s="4" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="L79" s="7" t="inlineStr">
         <is>
@@ -8828,7 +8828,7 @@
         <v>0</v>
       </c>
       <c r="V79" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W79" s="9" t="n">
         <v>0</v>
@@ -8884,13 +8884,13 @@
         </is>
       </c>
       <c r="I80" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="J80" s="4" t="n">
         <v>10</v>
       </c>
       <c r="K80" s="4" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="L80" s="7" t="inlineStr">
         <is>
@@ -8985,13 +8985,13 @@
         </is>
       </c>
       <c r="I81" s="4" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="J81" s="4" t="n">
         <v>16</v>
       </c>
       <c r="K81" s="4" t="n">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="L81" s="7" t="inlineStr">
         <is>
@@ -9086,13 +9086,13 @@
         </is>
       </c>
       <c r="I82" s="4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J82" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K82" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L82" s="7" t="inlineStr">
         <is>
@@ -9177,7 +9177,7 @@
         </is>
       </c>
       <c r="E83" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F83" s="6" t="n">
         <v>10</v>
@@ -9247,8 +9247,8 @@
       <c r="Y83" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="Z83" s="9" t="n">
-        <v>0</v>
+      <c r="Z83" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="AA83" s="10" t="n">
         <v>1</v>
@@ -9290,17 +9290,17 @@
         </is>
       </c>
       <c r="I84" s="4" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="J84" s="4" t="n">
         <v>22</v>
       </c>
       <c r="K84" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L84" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-8</v>
+      </c>
+      <c r="L84" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M84" s="8" t="n">
@@ -9391,17 +9391,17 @@
         </is>
       </c>
       <c r="I85" s="4" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="J85" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K85" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L85" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-5</v>
+      </c>
+      <c r="L85" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M85" s="8" t="n">
@@ -9496,17 +9496,17 @@
         </is>
       </c>
       <c r="I86" s="4" t="n">
-        <v>48</v>
+        <v>13</v>
       </c>
       <c r="J86" s="4" t="n">
         <v>41</v>
       </c>
       <c r="K86" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="L86" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-28</v>
+      </c>
+      <c r="L86" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M86" s="8" t="n">
@@ -9601,13 +9601,13 @@
         </is>
       </c>
       <c r="I87" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J87" s="4" t="n">
         <v>5</v>
       </c>
       <c r="K87" s="4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="L87" s="7" t="inlineStr">
         <is>
@@ -9702,13 +9702,13 @@
         </is>
       </c>
       <c r="I88" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="J88" s="4" t="n">
         <v>14</v>
       </c>
       <c r="K88" s="4" t="n">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="L88" s="7" t="inlineStr">
         <is>
@@ -9803,17 +9803,17 @@
         </is>
       </c>
       <c r="I89" s="4" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="J89" s="4" t="n">
         <v>22</v>
       </c>
       <c r="K89" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L89" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-9</v>
+      </c>
+      <c r="L89" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M89" s="8" t="n">
@@ -9904,13 +9904,13 @@
         </is>
       </c>
       <c r="I90" s="4" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="J90" s="4" t="n">
         <v>25</v>
       </c>
       <c r="K90" s="4" t="n">
-        <v>6</v>
+        <v>-3</v>
       </c>
       <c r="L90" s="4" t="inlineStr">
         <is>
@@ -10009,17 +10009,17 @@
         </is>
       </c>
       <c r="I91" s="4" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="J91" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K91" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L91" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-6</v>
+      </c>
+      <c r="L91" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M91" s="8" t="n">
@@ -10054,7 +10054,7 @@
         <v>0</v>
       </c>
       <c r="V91" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W91" s="9" t="n">
         <v>0</v>
@@ -10110,13 +10110,13 @@
         </is>
       </c>
       <c r="I92" s="4" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="J92" s="4" t="n">
         <v>12</v>
       </c>
       <c r="K92" s="4" t="n">
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="L92" s="7" t="inlineStr">
         <is>
@@ -10211,17 +10211,17 @@
         </is>
       </c>
       <c r="I93" s="4" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="J93" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K93" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L93" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-4</v>
+      </c>
+      <c r="L93" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M93" s="8" t="n">
@@ -10316,13 +10316,13 @@
         </is>
       </c>
       <c r="I94" s="4" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="J94" s="4" t="n">
         <v>27</v>
       </c>
       <c r="K94" s="4" t="n">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="L94" s="4" t="inlineStr">
         <is>
@@ -10407,7 +10407,7 @@
         </is>
       </c>
       <c r="E95" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F95" s="6" t="n">
         <v>10</v>
@@ -10421,17 +10421,17 @@
         </is>
       </c>
       <c r="I95" s="4" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="J95" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K95" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L95" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-4</v>
+      </c>
+      <c r="L95" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M95" s="8" t="n">
@@ -10465,11 +10465,11 @@
       <c r="U95" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="V95" s="9" t="n">
-        <v>2</v>
+      <c r="V95" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="W95" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X95" s="10" t="n">
         <v>6</v>
@@ -10526,13 +10526,13 @@
         </is>
       </c>
       <c r="I96" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J96" s="4" t="n">
         <v>14</v>
       </c>
       <c r="K96" s="4" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="L96" s="7" t="inlineStr">
         <is>
@@ -10553,7 +10553,7 @@
         </is>
       </c>
       <c r="P96" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q96" s="9" t="n">
         <v>0</v>
@@ -10627,13 +10627,13 @@
         </is>
       </c>
       <c r="I97" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J97" s="4" t="n">
         <v>14</v>
       </c>
       <c r="K97" s="4" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="L97" s="7" t="inlineStr">
         <is>
@@ -10728,13 +10728,13 @@
         </is>
       </c>
       <c r="I98" s="4" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="J98" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K98" s="4" t="n">
-        <v>1</v>
+        <v>-11</v>
       </c>
       <c r="L98" s="7" t="inlineStr">
         <is>
@@ -10829,13 +10829,13 @@
         </is>
       </c>
       <c r="I99" s="4" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="J99" s="4" t="n">
         <v>13</v>
       </c>
       <c r="K99" s="4" t="n">
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="L99" s="7" t="inlineStr">
         <is>
@@ -10930,17 +10930,17 @@
         </is>
       </c>
       <c r="I100" s="4" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="J100" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K100" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L100" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-6</v>
+      </c>
+      <c r="L100" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M100" s="8" t="n">
@@ -10975,7 +10975,7 @@
         <v>0</v>
       </c>
       <c r="V100" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W100" s="9" t="n">
         <v>0</v>
@@ -11021,7 +11021,7 @@
         </is>
       </c>
       <c r="E101" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F101" s="6" t="n">
         <v>10</v>
@@ -11079,11 +11079,11 @@
       <c r="U101" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="V101" s="9" t="n">
-        <v>2</v>
+      <c r="V101" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="W101" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X101" s="10" t="n">
         <v>4</v>
@@ -11126,7 +11126,7 @@
         </is>
       </c>
       <c r="E102" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F102" s="6" t="n">
         <v>10</v>
@@ -11140,13 +11140,13 @@
         </is>
       </c>
       <c r="I102" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="J102" s="4" t="n">
         <v>18</v>
       </c>
       <c r="K102" s="4" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="L102" s="7" t="inlineStr">
         <is>
@@ -11175,8 +11175,8 @@
       <c r="R102" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="S102" s="9" t="n">
-        <v>0</v>
+      <c r="S102" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="T102" s="9" t="n">
         <v>0</v>
@@ -11332,7 +11332,7 @@
         </is>
       </c>
       <c r="E104" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F104" s="6" t="n">
         <v>10</v>
@@ -11346,13 +11346,13 @@
         </is>
       </c>
       <c r="I104" s="4" t="n">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="J104" s="4" t="n">
         <v>40</v>
       </c>
       <c r="K104" s="4" t="n">
-        <v>5</v>
+        <v>-6</v>
       </c>
       <c r="L104" s="4" t="inlineStr">
         <is>
@@ -11393,8 +11393,8 @@
       <c r="V104" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="W104" s="9" t="n">
-        <v>1</v>
+      <c r="W104" s="10" t="n">
+        <v>5</v>
       </c>
       <c r="X104" s="10" t="n">
         <v>7</v>
@@ -11451,13 +11451,13 @@
         </is>
       </c>
       <c r="I105" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J105" s="4" t="n">
         <v>19</v>
       </c>
       <c r="K105" s="4" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="L105" s="7" t="inlineStr">
         <is>
@@ -11496,7 +11496,7 @@
         <v>1</v>
       </c>
       <c r="V105" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W105" s="9" t="n">
         <v>0</v>
@@ -11556,13 +11556,13 @@
         </is>
       </c>
       <c r="I106" s="4" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="J106" s="4" t="n">
         <v>16</v>
       </c>
       <c r="K106" s="4" t="n">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="L106" s="7" t="inlineStr">
         <is>
@@ -11601,7 +11601,7 @@
         <v>0</v>
       </c>
       <c r="V106" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W106" s="9" t="n">
         <v>0</v>
@@ -11657,13 +11657,13 @@
         </is>
       </c>
       <c r="I107" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="J107" s="4" t="n">
         <v>16</v>
       </c>
       <c r="K107" s="4" t="n">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="L107" s="7" t="inlineStr">
         <is>
@@ -11702,7 +11702,7 @@
         <v>0</v>
       </c>
       <c r="V107" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W107" s="9" t="n">
         <v>0</v>
@@ -11758,13 +11758,13 @@
         </is>
       </c>
       <c r="I108" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J108" s="4" t="n">
         <v>9</v>
       </c>
       <c r="K108" s="4" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="L108" s="7" t="inlineStr">
         <is>
@@ -11845,7 +11845,7 @@
         </is>
       </c>
       <c r="E109" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F109" s="6" t="n">
         <v>10</v>
@@ -11859,17 +11859,17 @@
         </is>
       </c>
       <c r="I109" s="4" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="J109" s="4" t="n">
         <v>21</v>
       </c>
       <c r="K109" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L109" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-2</v>
+      </c>
+      <c r="L109" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M109" s="8" t="n">
@@ -11903,8 +11903,8 @@
       <c r="U109" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="V109" s="9" t="n">
-        <v>3</v>
+      <c r="V109" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="W109" s="9" t="n">
         <v>0</v>
@@ -11964,17 +11964,17 @@
         </is>
       </c>
       <c r="I110" s="4" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="J110" s="4" t="n">
         <v>27</v>
       </c>
       <c r="K110" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L110" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-15</v>
+      </c>
+      <c r="L110" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M110" s="8" t="n">
@@ -12009,7 +12009,7 @@
         <v>0</v>
       </c>
       <c r="V110" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W110" s="9" t="n">
         <v>0</v>
@@ -12069,13 +12069,13 @@
         </is>
       </c>
       <c r="I111" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="J111" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K111" s="4" t="n">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="L111" s="7" t="inlineStr">
         <is>
@@ -12170,13 +12170,13 @@
         </is>
       </c>
       <c r="I112" s="4" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="J112" s="4" t="n">
         <v>25</v>
       </c>
       <c r="K112" s="4" t="n">
-        <v>6</v>
+        <v>-2</v>
       </c>
       <c r="L112" s="4" t="inlineStr">
         <is>
@@ -12218,7 +12218,7 @@
         <v>4</v>
       </c>
       <c r="W112" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X112" s="10" t="n">
         <v>7</v>
@@ -12275,13 +12275,13 @@
         </is>
       </c>
       <c r="I113" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J113" s="4" t="n">
         <v>7</v>
       </c>
       <c r="K113" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L113" s="7" t="inlineStr">
         <is>
@@ -12320,7 +12320,7 @@
         <v>0</v>
       </c>
       <c r="V113" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W113" s="9" t="n">
         <v>0</v>
@@ -12477,17 +12477,17 @@
         </is>
       </c>
       <c r="I115" s="4" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="J115" s="4" t="n">
         <v>21</v>
       </c>
       <c r="K115" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L115" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-11</v>
+      </c>
+      <c r="L115" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M115" s="8" t="n">
@@ -12568,7 +12568,7 @@
         </is>
       </c>
       <c r="E116" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F116" s="6" t="n">
         <v>10</v>
@@ -12582,17 +12582,17 @@
         </is>
       </c>
       <c r="I116" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J116" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K116" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L116" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-2</v>
+      </c>
+      <c r="L116" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M116" s="8" t="n">
@@ -12617,8 +12617,8 @@
       <c r="R116" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="S116" s="9" t="n">
-        <v>1</v>
+      <c r="S116" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="T116" s="10" t="n">
         <v>1</v>
@@ -12687,13 +12687,13 @@
         </is>
       </c>
       <c r="I117" s="4" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="J117" s="4" t="n">
         <v>15</v>
       </c>
       <c r="K117" s="4" t="n">
-        <v>1</v>
+        <v>-5</v>
       </c>
       <c r="L117" s="7" t="inlineStr">
         <is>
@@ -12788,13 +12788,13 @@
         </is>
       </c>
       <c r="I118" s="4" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="J118" s="4" t="n">
         <v>18</v>
       </c>
       <c r="K118" s="4" t="n">
-        <v>0</v>
+        <v>-17</v>
       </c>
       <c r="L118" s="7" t="inlineStr">
         <is>
@@ -12889,13 +12889,13 @@
         </is>
       </c>
       <c r="I119" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="J119" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K119" s="4" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="L119" s="7" t="inlineStr">
         <is>
@@ -12994,17 +12994,17 @@
         </is>
       </c>
       <c r="I120" s="4" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="J120" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K120" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L120" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-3</v>
+      </c>
+      <c r="L120" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M120" s="8" t="n">
@@ -13099,13 +13099,13 @@
         </is>
       </c>
       <c r="I121" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J121" s="4" t="n">
         <v>9</v>
       </c>
       <c r="K121" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L121" s="7" t="inlineStr">
         <is>
@@ -13245,7 +13245,7 @@
         <v>0</v>
       </c>
       <c r="V122" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W122" s="9" t="n">
         <v>0</v>
@@ -13301,13 +13301,13 @@
         </is>
       </c>
       <c r="I123" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J123" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K123" s="4" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="L123" s="7" t="inlineStr">
         <is>
@@ -13501,13 +13501,13 @@
         </is>
       </c>
       <c r="I125" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J125" s="4" t="n">
         <v>8</v>
       </c>
       <c r="K125" s="4" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="L125" s="7" t="inlineStr">
         <is>
@@ -13602,13 +13602,13 @@
         </is>
       </c>
       <c r="I126" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J126" s="4" t="n">
         <v>14</v>
       </c>
       <c r="K126" s="4" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="L126" s="7" t="inlineStr">
         <is>
@@ -13629,7 +13629,7 @@
         </is>
       </c>
       <c r="P126" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q126" s="9" t="n">
         <v>1</v>
@@ -13703,13 +13703,13 @@
         </is>
       </c>
       <c r="I127" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J127" s="4" t="n">
         <v>9</v>
       </c>
       <c r="K127" s="4" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="L127" s="7" t="inlineStr">
         <is>
@@ -13909,13 +13909,13 @@
         </is>
       </c>
       <c r="I129" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="J129" s="4" t="n">
         <v>13</v>
       </c>
       <c r="K129" s="4" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="L129" s="7" t="inlineStr">
         <is>
@@ -13945,7 +13945,7 @@
         <v>0</v>
       </c>
       <c r="S129" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T129" s="9" t="n">
         <v>0</v>
@@ -13954,7 +13954,7 @@
         <v>0</v>
       </c>
       <c r="V129" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W129" s="9" t="n">
         <v>0</v>
@@ -14010,13 +14010,13 @@
         </is>
       </c>
       <c r="I130" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J130" s="4" t="n">
         <v>6</v>
       </c>
       <c r="K130" s="4" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="L130" s="7" t="inlineStr">
         <is>
@@ -14046,7 +14046,7 @@
         <v>0</v>
       </c>
       <c r="S130" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T130" s="9" t="n">
         <v>0</v>
@@ -14111,17 +14111,17 @@
         </is>
       </c>
       <c r="I131" s="4" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="J131" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K131" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="L131" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>1</v>
+      </c>
+      <c r="L131" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M131" s="8" t="n">
@@ -14159,7 +14159,7 @@
         <v>4</v>
       </c>
       <c r="W131" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X131" s="10" t="n">
         <v>5</v>
@@ -14212,13 +14212,13 @@
         </is>
       </c>
       <c r="I132" s="4" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="J132" s="4" t="n">
         <v>26</v>
       </c>
       <c r="K132" s="4" t="n">
-        <v>4</v>
+        <v>-5</v>
       </c>
       <c r="L132" s="4" t="inlineStr">
         <is>
@@ -14317,13 +14317,13 @@
         </is>
       </c>
       <c r="I133" s="4" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="J133" s="4" t="n">
         <v>27</v>
       </c>
       <c r="K133" s="4" t="n">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="L133" s="4" t="inlineStr">
         <is>
@@ -14362,7 +14362,7 @@
         <v>1</v>
       </c>
       <c r="V133" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W133" s="9" t="n">
         <v>0</v>
@@ -14467,7 +14467,7 @@
         <v>0</v>
       </c>
       <c r="V134" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W134" s="9" t="n">
         <v>0</v>
@@ -14523,17 +14523,17 @@
         </is>
       </c>
       <c r="I135" s="4" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="J135" s="4" t="n">
         <v>21</v>
       </c>
       <c r="K135" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L135" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-7</v>
+      </c>
+      <c r="L135" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M135" s="8" t="n">
@@ -14628,17 +14628,17 @@
         </is>
       </c>
       <c r="I136" s="4" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="J136" s="4" t="n">
         <v>24</v>
       </c>
       <c r="K136" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L136" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-13</v>
+      </c>
+      <c r="L136" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M136" s="8" t="n">
@@ -14733,13 +14733,13 @@
         </is>
       </c>
       <c r="I137" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J137" s="4" t="n">
         <v>7</v>
       </c>
       <c r="K137" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L137" s="7" t="inlineStr">
         <is>
@@ -14778,7 +14778,7 @@
         <v>0</v>
       </c>
       <c r="V137" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W137" s="9" t="n">
         <v>0</v>
@@ -14834,17 +14834,17 @@
         </is>
       </c>
       <c r="I138" s="4" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="J138" s="4" t="n">
         <v>22</v>
       </c>
       <c r="K138" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L138" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-9</v>
+      </c>
+      <c r="L138" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M138" s="8" t="n">
@@ -14876,7 +14876,7 @@
         <v>1</v>
       </c>
       <c r="U138" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V138" s="9" t="n">
         <v>0</v>
@@ -15040,13 +15040,13 @@
         </is>
       </c>
       <c r="I140" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J140" s="4" t="n">
         <v>12</v>
       </c>
       <c r="K140" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L140" s="7" t="inlineStr">
         <is>
@@ -15141,17 +15141,17 @@
         </is>
       </c>
       <c r="I141" s="4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="J141" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K141" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L141" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-5</v>
+      </c>
+      <c r="L141" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M141" s="8" t="n">
@@ -15246,17 +15246,17 @@
         </is>
       </c>
       <c r="I142" s="4" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="J142" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K142" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L142" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-9</v>
+      </c>
+      <c r="L142" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M142" s="8" t="n">
@@ -15291,7 +15291,7 @@
         <v>0</v>
       </c>
       <c r="V142" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W142" s="9" t="n">
         <v>0</v>
@@ -15347,13 +15347,13 @@
         </is>
       </c>
       <c r="I143" s="4" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="J143" s="4" t="n">
         <v>15</v>
       </c>
       <c r="K143" s="4" t="n">
-        <v>1</v>
+        <v>-6</v>
       </c>
       <c r="L143" s="7" t="inlineStr">
         <is>
@@ -15448,17 +15448,17 @@
         </is>
       </c>
       <c r="I144" s="4" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="J144" s="4" t="n">
         <v>24</v>
       </c>
       <c r="K144" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L144" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-9</v>
+      </c>
+      <c r="L144" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M144" s="8" t="n">
@@ -15553,13 +15553,13 @@
         </is>
       </c>
       <c r="I145" s="4" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="J145" s="4" t="n">
         <v>28</v>
       </c>
       <c r="K145" s="4" t="n">
-        <v>1</v>
+        <v>-5</v>
       </c>
       <c r="L145" s="4" t="inlineStr">
         <is>
@@ -15598,7 +15598,7 @@
         <v>1</v>
       </c>
       <c r="V145" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W145" s="9" t="n">
         <v>0</v>
@@ -15644,7 +15644,7 @@
         </is>
       </c>
       <c r="E146" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F146" s="6" t="n">
         <v>10</v>
@@ -15658,13 +15658,13 @@
         </is>
       </c>
       <c r="I146" s="4" t="n">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="J146" s="4" t="n">
         <v>34</v>
       </c>
       <c r="K146" s="4" t="n">
-        <v>3</v>
+        <v>-7</v>
       </c>
       <c r="L146" s="4" t="inlineStr">
         <is>
@@ -15685,7 +15685,7 @@
         </is>
       </c>
       <c r="P146" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q146" s="9" t="n">
         <v>0</v>
@@ -15702,8 +15702,8 @@
       <c r="U146" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="V146" s="9" t="n">
-        <v>3</v>
+      <c r="V146" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="W146" s="9" t="n">
         <v>0</v>
@@ -15763,13 +15763,13 @@
         </is>
       </c>
       <c r="I147" s="4" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="J147" s="4" t="n">
         <v>15</v>
       </c>
       <c r="K147" s="4" t="n">
-        <v>4</v>
+        <v>-2</v>
       </c>
       <c r="L147" s="7" t="inlineStr">
         <is>
@@ -15790,7 +15790,7 @@
         </is>
       </c>
       <c r="P147" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q147" s="9" t="n">
         <v>0</v>
@@ -15811,7 +15811,7 @@
         <v>4</v>
       </c>
       <c r="W147" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X147" s="10" t="n">
         <v>7</v>
@@ -15868,13 +15868,13 @@
         </is>
       </c>
       <c r="I148" s="4" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="J148" s="4" t="n">
         <v>19</v>
       </c>
       <c r="K148" s="4" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="L148" s="7" t="inlineStr">
         <is>
@@ -15973,13 +15973,13 @@
         </is>
       </c>
       <c r="I149" s="4" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="J149" s="4" t="n">
         <v>16</v>
       </c>
       <c r="K149" s="4" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="L149" s="7" t="inlineStr">
         <is>
@@ -16074,17 +16074,17 @@
         </is>
       </c>
       <c r="I150" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="J150" s="4" t="n">
         <v>18</v>
       </c>
       <c r="K150" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="L150" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>0</v>
+      </c>
+      <c r="L150" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M150" s="8" t="n">
@@ -16179,13 +16179,13 @@
         </is>
       </c>
       <c r="I151" s="4" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="J151" s="4" t="n">
         <v>14</v>
       </c>
       <c r="K151" s="4" t="n">
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="L151" s="7" t="inlineStr">
         <is>
@@ -16284,13 +16284,13 @@
         </is>
       </c>
       <c r="I152" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="J152" s="4" t="n">
         <v>14</v>
       </c>
       <c r="K152" s="4" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="L152" s="7" t="inlineStr">
         <is>
@@ -16385,17 +16385,17 @@
         </is>
       </c>
       <c r="I153" s="4" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="J153" s="4" t="n">
         <v>25</v>
       </c>
       <c r="K153" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L153" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-11</v>
+      </c>
+      <c r="L153" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M153" s="8" t="n">
@@ -16430,7 +16430,7 @@
         <v>0</v>
       </c>
       <c r="V153" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W153" s="9" t="n">
         <v>0</v>
@@ -16490,13 +16490,13 @@
         </is>
       </c>
       <c r="I154" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J154" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K154" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L154" s="7" t="inlineStr">
         <is>
@@ -16523,7 +16523,7 @@
         <v>2</v>
       </c>
       <c r="R154" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S154" s="9" t="n">
         <v>1</v>
@@ -16535,7 +16535,7 @@
         <v>0</v>
       </c>
       <c r="V154" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W154" s="9" t="n">
         <v>0</v>
@@ -16700,17 +16700,17 @@
         </is>
       </c>
       <c r="I156" s="4" t="n">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="J156" s="4" t="n">
         <v>25</v>
       </c>
       <c r="K156" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="L156" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-7</v>
+      </c>
+      <c r="L156" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M156" s="8" t="n">
@@ -16748,7 +16748,7 @@
         <v>4</v>
       </c>
       <c r="W156" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X156" s="10" t="n">
         <v>4</v>
@@ -16805,13 +16805,13 @@
         </is>
       </c>
       <c r="I157" s="4" t="n">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="J157" s="4" t="n">
         <v>37</v>
       </c>
       <c r="K157" s="4" t="n">
-        <v>3</v>
+        <v>-4</v>
       </c>
       <c r="L157" s="4" t="inlineStr">
         <is>
@@ -16910,13 +16910,13 @@
         </is>
       </c>
       <c r="I158" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J158" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K158" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L158" s="7" t="inlineStr">
         <is>
@@ -16955,7 +16955,7 @@
         <v>0</v>
       </c>
       <c r="V158" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W158" s="9" t="n">
         <v>0</v>
@@ -17011,17 +17011,17 @@
         </is>
       </c>
       <c r="I159" s="4" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="J159" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K159" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L159" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-12</v>
+      </c>
+      <c r="L159" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M159" s="8" t="n">
@@ -17038,7 +17038,7 @@
         </is>
       </c>
       <c r="P159" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q159" s="9" t="n">
         <v>1</v>
@@ -17116,17 +17116,17 @@
         </is>
       </c>
       <c r="I160" s="4" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="J160" s="4" t="n">
         <v>26</v>
       </c>
       <c r="K160" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L160" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-9</v>
+      </c>
+      <c r="L160" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M160" s="8" t="n">
@@ -17161,7 +17161,7 @@
         <v>0</v>
       </c>
       <c r="V160" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W160" s="9" t="n">
         <v>0</v>
@@ -17221,13 +17221,13 @@
         </is>
       </c>
       <c r="I161" s="4" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="J161" s="4" t="n">
         <v>13</v>
       </c>
       <c r="K161" s="4" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="L161" s="7" t="inlineStr">
         <is>
@@ -17322,13 +17322,13 @@
         </is>
       </c>
       <c r="I162" s="4" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="J162" s="4" t="n">
         <v>28</v>
       </c>
       <c r="K162" s="4" t="n">
-        <v>1</v>
+        <v>-6</v>
       </c>
       <c r="L162" s="4" t="inlineStr">
         <is>
@@ -17367,7 +17367,7 @@
         <v>1</v>
       </c>
       <c r="V162" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W162" s="9" t="n">
         <v>0</v>
@@ -17427,17 +17427,17 @@
         </is>
       </c>
       <c r="I163" s="4" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="J163" s="4" t="n">
         <v>27</v>
       </c>
       <c r="K163" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L163" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-14</v>
+      </c>
+      <c r="L163" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M163" s="8" t="n">
@@ -17518,7 +17518,7 @@
         </is>
       </c>
       <c r="E164" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F164" s="6" t="n">
         <v>10</v>
@@ -17532,17 +17532,17 @@
         </is>
       </c>
       <c r="I164" s="4" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="J164" s="4" t="n">
         <v>19</v>
       </c>
       <c r="K164" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L164" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-5</v>
+      </c>
+      <c r="L164" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M164" s="8" t="n">
@@ -17576,11 +17576,11 @@
       <c r="U164" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="V164" s="9" t="n">
+      <c r="V164" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="W164" s="9" t="n">
         <v>2</v>
-      </c>
-      <c r="W164" s="9" t="n">
-        <v>0</v>
       </c>
       <c r="X164" s="10" t="n">
         <v>7</v>
@@ -17637,13 +17637,13 @@
         </is>
       </c>
       <c r="I165" s="4" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="J165" s="4" t="n">
         <v>15</v>
       </c>
       <c r="K165" s="4" t="n">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="L165" s="7" t="inlineStr">
         <is>
@@ -17738,13 +17738,13 @@
         </is>
       </c>
       <c r="I166" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J166" s="4" t="n">
         <v>8</v>
       </c>
       <c r="K166" s="4" t="n">
-        <v>1</v>
+        <v>-7</v>
       </c>
       <c r="L166" s="7" t="inlineStr">
         <is>
@@ -17839,13 +17839,13 @@
         </is>
       </c>
       <c r="I167" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J167" s="4" t="n">
         <v>10</v>
       </c>
       <c r="K167" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L167" s="7" t="inlineStr">
         <is>
@@ -17940,13 +17940,13 @@
         </is>
       </c>
       <c r="I168" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J168" s="4" t="n">
         <v>9</v>
       </c>
       <c r="K168" s="4" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="L168" s="7" t="inlineStr">
         <is>
@@ -18041,13 +18041,13 @@
         </is>
       </c>
       <c r="I169" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="J169" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K169" s="4" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="L169" s="7" t="inlineStr">
         <is>
@@ -18086,7 +18086,7 @@
         <v>0</v>
       </c>
       <c r="V169" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W169" s="9" t="n">
         <v>0</v>
@@ -18132,7 +18132,7 @@
         </is>
       </c>
       <c r="E170" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F170" s="6" t="n">
         <v>10</v>
@@ -18146,13 +18146,13 @@
         </is>
       </c>
       <c r="I170" s="4" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J170" s="4" t="n">
         <v>14</v>
       </c>
       <c r="K170" s="4" t="n">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="L170" s="7" t="inlineStr">
         <is>
@@ -18184,14 +18184,14 @@
       <c r="S170" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="T170" s="9" t="n">
-        <v>0</v>
+      <c r="T170" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="U170" s="9" t="n">
         <v>0</v>
       </c>
       <c r="V170" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W170" s="9" t="n">
         <v>0</v>
@@ -18296,7 +18296,7 @@
         <v>0</v>
       </c>
       <c r="V171" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W171" s="9" t="n">
         <v>0</v>
@@ -18352,13 +18352,13 @@
         </is>
       </c>
       <c r="I172" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="J172" s="4" t="n">
         <v>10</v>
       </c>
       <c r="K172" s="4" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="L172" s="7" t="inlineStr">
         <is>
@@ -18453,13 +18453,13 @@
         </is>
       </c>
       <c r="I173" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J173" s="4" t="n">
         <v>9</v>
       </c>
       <c r="K173" s="4" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="L173" s="7" t="inlineStr">
         <is>
@@ -18498,7 +18498,7 @@
         <v>0</v>
       </c>
       <c r="V173" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W173" s="9" t="n">
         <v>0</v>
@@ -18554,13 +18554,13 @@
         </is>
       </c>
       <c r="I174" s="4" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="J174" s="4" t="n">
         <v>16</v>
       </c>
       <c r="K174" s="4" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="L174" s="7" t="inlineStr">
         <is>
@@ -18655,13 +18655,13 @@
         </is>
       </c>
       <c r="I175" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="J175" s="4" t="n">
         <v>15</v>
       </c>
       <c r="K175" s="4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="L175" s="7" t="inlineStr">
         <is>
@@ -18700,7 +18700,7 @@
         <v>0</v>
       </c>
       <c r="V175" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W175" s="9" t="n">
         <v>0</v>
@@ -18756,17 +18756,17 @@
         </is>
       </c>
       <c r="I176" s="4" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="J176" s="4" t="n">
         <v>25</v>
       </c>
       <c r="K176" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L176" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-11</v>
+      </c>
+      <c r="L176" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M176" s="8" t="n">
@@ -18861,13 +18861,13 @@
         </is>
       </c>
       <c r="I177" s="4" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="J177" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K177" s="4" t="n">
-        <v>1</v>
+        <v>-5</v>
       </c>
       <c r="L177" s="7" t="inlineStr">
         <is>
@@ -19067,17 +19067,17 @@
         </is>
       </c>
       <c r="I179" s="4" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="J179" s="4" t="n">
         <v>16</v>
       </c>
       <c r="K179" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L179" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-6</v>
+      </c>
+      <c r="L179" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M179" s="8" t="n">
@@ -19172,17 +19172,17 @@
         </is>
       </c>
       <c r="I180" s="4" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="J180" s="4" t="n">
         <v>21</v>
       </c>
       <c r="K180" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L180" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-7</v>
+      </c>
+      <c r="L180" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M180" s="8" t="n">
@@ -19217,7 +19217,7 @@
         <v>2</v>
       </c>
       <c r="V180" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W180" s="9" t="n">
         <v>0</v>
@@ -19277,13 +19277,13 @@
         </is>
       </c>
       <c r="I181" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="J181" s="4" t="n">
         <v>13</v>
       </c>
       <c r="K181" s="4" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="L181" s="7" t="inlineStr">
         <is>
@@ -19382,17 +19382,17 @@
         </is>
       </c>
       <c r="I182" s="4" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="J182" s="4" t="n">
         <v>20</v>
       </c>
       <c r="K182" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L182" s="4" t="inlineStr">
-        <is>
-          <t>yes</t>
+        <v>-5</v>
+      </c>
+      <c r="L182" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
       <c r="M182" s="8" t="n">
@@ -19487,13 +19487,13 @@
         </is>
       </c>
       <c r="I183" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="J183" s="4" t="n">
         <v>8</v>
       </c>
       <c r="K183" s="4" t="n">
-        <v>1</v>
+        <v>-4</v>
       </c>
       <c r="L183" s="7" t="inlineStr">
         <is>
@@ -19588,13 +19588,13 @@
         </is>
       </c>
       <c r="I184" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J184" s="4" t="n">
         <v>8</v>
       </c>
       <c r="K184" s="4" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="L184" s="7" t="inlineStr">
         <is>
@@ -19689,13 +19689,13 @@
         </is>
       </c>
       <c r="I185" s="4" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="J185" s="4" t="n">
         <v>18</v>
       </c>
       <c r="K185" s="4" t="n">
-        <v>0</v>
+        <v>-18</v>
       </c>
       <c r="L185" s="7" t="inlineStr">
         <is>
@@ -19859,7 +19859,7 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -19877,7 +19877,7 @@
         <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -19892,7 +19892,7 @@
         <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -19925,7 +19925,7 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -19991,7 +19991,7 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -20024,7 +20024,7 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -20057,7 +20057,7 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -20090,7 +20090,7 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -20123,7 +20123,7 @@
         <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -20141,7 +20141,7 @@
         <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -20189,7 +20189,7 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -20222,7 +20222,7 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -20240,7 +20240,7 @@
         <v>5</v>
       </c>
       <c r="D14" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -20321,7 +20321,7 @@
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -20339,7 +20339,7 @@
         <v>5</v>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -20354,7 +20354,7 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -20372,7 +20372,7 @@
         <v>7</v>
       </c>
       <c r="D18" t="n">
-        <v>1.43</v>
+        <v>1.57</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -20387,7 +20387,7 @@
         <v>1</v>
       </c>
       <c r="I18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -20405,7 +20405,7 @@
         <v>6</v>
       </c>
       <c r="D19" t="n">
-        <v>0.83</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -20420,7 +20420,7 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -20453,7 +20453,7 @@
         <v>1</v>
       </c>
       <c r="I20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -20471,7 +20471,7 @@
         <v>5</v>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -20486,7 +20486,7 @@
         <v>1</v>
       </c>
       <c r="I21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -20504,7 +20504,7 @@
         <v>5</v>
       </c>
       <c r="D22" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
@@ -20519,7 +20519,7 @@
         <v>1</v>
       </c>
       <c r="I22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -20537,7 +20537,7 @@
         <v>6</v>
       </c>
       <c r="D23" t="n">
-        <v>1.5</v>
+        <v>1.83</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -20570,13 +20570,13 @@
         <v>7</v>
       </c>
       <c r="D24" t="n">
-        <v>1.43</v>
+        <v>1.57</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -20585,7 +20585,7 @@
         <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -20603,7 +20603,7 @@
         <v>4</v>
       </c>
       <c r="D25" t="n">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -20618,7 +20618,7 @@
         <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -20651,7 +20651,7 @@
         <v>1</v>
       </c>
       <c r="I26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -20717,7 +20717,7 @@
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
@@ -20750,7 +20750,7 @@
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -20783,7 +20783,7 @@
         <v>1</v>
       </c>
       <c r="I30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -20801,7 +20801,7 @@
         <v>4</v>
       </c>
       <c r="D31" t="n">
-        <v>3.25</v>
+        <v>3.5</v>
       </c>
       <c r="E31" t="n">
         <v>1</v>
@@ -20816,7 +20816,7 @@
         <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
@@ -20849,7 +20849,7 @@
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -20882,7 +20882,7 @@
         <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -20915,7 +20915,7 @@
         <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -20933,7 +20933,7 @@
         <v>5</v>
       </c>
       <c r="D35" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
@@ -20948,7 +20948,7 @@
         <v>1</v>
       </c>
       <c r="I35" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -20966,7 +20966,7 @@
         <v>4</v>
       </c>
       <c r="D36" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
@@ -21014,7 +21014,7 @@
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -21047,7 +21047,7 @@
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -21080,7 +21080,7 @@
         <v>2</v>
       </c>
       <c r="I39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>